<commit_message>
Presidents contact file updated from predsjednici-01-10.xlsx.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/main/resources/documents/2026/predsjednici kontakt.xlsx
+++ b/src/main/resources/documents/2026/predsjednici kontakt.xlsx
@@ -1209,10 +1209,26 @@
           <t>Замjеник предсjедника</t>
         </is>
       </c>
-      <c r="C22" s="26" t="n"/>
-      <c r="D22" s="26" t="n"/>
-      <c r="E22" s="26" t="n"/>
-      <c r="F22" s="26" t="n"/>
+      <c r="C22" s="26" t="inlineStr">
+        <is>
+          <t>2304981105067</t>
+        </is>
+      </c>
+      <c r="D22" s="26" t="inlineStr">
+        <is>
+          <t>ДУШКА</t>
+        </is>
+      </c>
+      <c r="E22" s="26" t="inlineStr">
+        <is>
+          <t>ОЗРЕН</t>
+        </is>
+      </c>
+      <c r="F22" s="26" t="inlineStr">
+        <is>
+          <t>065/682-963</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -3531,22 +3547,22 @@
       </c>
       <c r="C99" s="26" t="inlineStr">
         <is>
-          <t>1002000105003</t>
+          <t>1408980105019</t>
         </is>
       </c>
       <c r="D99" s="26" t="inlineStr">
         <is>
-          <t>ДАJАНА</t>
+          <t>ЖАНА</t>
         </is>
       </c>
       <c r="E99" s="26" t="inlineStr">
         <is>
-          <t>ЂУКИЋ</t>
+          <t>БАБИЋ</t>
         </is>
       </c>
       <c r="F99" s="26" t="inlineStr">
         <is>
-          <t>066/818-877</t>
+          <t>066/788-888</t>
         </is>
       </c>
     </row>
@@ -3563,22 +3579,22 @@
       </c>
       <c r="C100" s="26" t="inlineStr">
         <is>
-          <t>2804963100034</t>
+          <t>1002000105003</t>
         </is>
       </c>
       <c r="D100" s="26" t="inlineStr">
         <is>
-          <t>ДРАШКО</t>
+          <t>ДАJАНА</t>
         </is>
       </c>
       <c r="E100" s="26" t="inlineStr">
         <is>
-          <t>ПЕJИЋ</t>
+          <t>ЂУКИЋ</t>
         </is>
       </c>
       <c r="F100" s="26" t="inlineStr">
         <is>
-          <t>065/342-002</t>
+          <t>066/818-877</t>
         </is>
       </c>
     </row>
@@ -5896,7 +5912,11 @@
           <t>БАJИЧИЋ</t>
         </is>
       </c>
-      <c r="F175" s="26" t="n"/>
+      <c r="F175" s="26" t="inlineStr">
+        <is>
+          <t>065/875-852</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="18" customHeight="1">
       <c r="A176" s="26" t="inlineStr">
@@ -8935,22 +8955,22 @@
       </c>
       <c r="C273" s="26" t="inlineStr">
         <is>
-          <t>1408980105019</t>
+          <t>1704957170006</t>
         </is>
       </c>
       <c r="D273" s="26" t="inlineStr">
         <is>
-          <t>ЖАНА</t>
+          <t>ХАЏИ МИЛЕНКО</t>
         </is>
       </c>
       <c r="E273" s="26" t="inlineStr">
         <is>
-          <t>БАБИЋ</t>
+          <t>ГАВРИЋ</t>
         </is>
       </c>
       <c r="F273" s="26" t="inlineStr">
         <is>
-          <t>066/788-888</t>
+          <t>065/474-121</t>
         </is>
       </c>
     </row>
@@ -9413,26 +9433,10 @@
           <t>Замjеник предсjедника</t>
         </is>
       </c>
-      <c r="C288" s="26" t="inlineStr">
-        <is>
-          <t>1704957170006</t>
-        </is>
-      </c>
-      <c r="D288" s="26" t="inlineStr">
-        <is>
-          <t>ХАЏИ МИЛЕНКО</t>
-        </is>
-      </c>
-      <c r="E288" s="26" t="inlineStr">
-        <is>
-          <t>ГАВРИЋ</t>
-        </is>
-      </c>
-      <c r="F288" s="26" t="inlineStr">
-        <is>
-          <t>065/474-121</t>
-        </is>
-      </c>
+      <c r="C288" s="26" t="n"/>
+      <c r="D288" s="26" t="n"/>
+      <c r="E288" s="26" t="n"/>
+      <c r="F288" s="26" t="n"/>
     </row>
     <row r="289" ht="18" customHeight="1">
       <c r="A289" s="26" t="inlineStr">
@@ -11335,22 +11339,22 @@
       </c>
       <c r="C351" s="26" t="inlineStr">
         <is>
-          <t>2409974107085</t>
+          <t>2804963100034</t>
         </is>
       </c>
       <c r="D351" s="26" t="inlineStr">
         <is>
-          <t>ДРАГАНА</t>
+          <t>ДРАШКО</t>
         </is>
       </c>
       <c r="E351" s="26" t="inlineStr">
         <is>
-          <t>АЋИЋ</t>
+          <t>ПЕJИЋ</t>
         </is>
       </c>
       <c r="F351" s="26" t="inlineStr">
         <is>
-          <t>065/603-179</t>
+          <t>065/342-002</t>
         </is>
       </c>
     </row>
@@ -14037,10 +14041,26 @@
           <t>Предсjедник</t>
         </is>
       </c>
-      <c r="C439" s="26" t="n"/>
-      <c r="D439" s="26" t="n"/>
-      <c r="E439" s="26" t="n"/>
-      <c r="F439" s="26" t="n"/>
+      <c r="C439" s="26" t="inlineStr">
+        <is>
+          <t>0907992105017</t>
+        </is>
+      </c>
+      <c r="D439" s="26" t="inlineStr">
+        <is>
+          <t>ВАЊА</t>
+        </is>
+      </c>
+      <c r="E439" s="26" t="inlineStr">
+        <is>
+          <t>JОВАНИЋ</t>
+        </is>
+      </c>
+      <c r="F439" s="26" t="inlineStr">
+        <is>
+          <t>065/001-001</t>
+        </is>
+      </c>
     </row>
     <row r="440" ht="18" customHeight="1">
       <c r="A440" s="26" t="inlineStr">
@@ -14053,26 +14073,10 @@
           <t>Замjеник предсjедника</t>
         </is>
       </c>
-      <c r="C440" s="26" t="inlineStr">
-        <is>
-          <t>0907992105017</t>
-        </is>
-      </c>
-      <c r="D440" s="26" t="inlineStr">
-        <is>
-          <t>ВАЊА</t>
-        </is>
-      </c>
-      <c r="E440" s="26" t="inlineStr">
-        <is>
-          <t>JОВАНИЋ</t>
-        </is>
-      </c>
-      <c r="F440" s="26" t="inlineStr">
-        <is>
-          <t>065/001-001</t>
-        </is>
-      </c>
+      <c r="C440" s="26" t="n"/>
+      <c r="D440" s="26" t="n"/>
+      <c r="E440" s="26" t="n"/>
+      <c r="F440" s="26" t="n"/>
     </row>
     <row r="441" ht="18" customHeight="1">
       <c r="A441" s="26" t="inlineStr">
@@ -16081,9 +16085,21 @@
           <t>Замjеник предсjедника</t>
         </is>
       </c>
-      <c r="C508" s="26" t="n"/>
-      <c r="D508" s="26" t="n"/>
-      <c r="E508" s="26" t="n"/>
+      <c r="C508" s="26" t="inlineStr">
+        <is>
+          <t>0802983105016</t>
+        </is>
+      </c>
+      <c r="D508" s="26" t="inlineStr">
+        <is>
+          <t>ДРАГАНА</t>
+        </is>
+      </c>
+      <c r="E508" s="26" t="inlineStr">
+        <is>
+          <t>МАСТАЛИЦА</t>
+        </is>
+      </c>
       <c r="F508" s="26" t="n"/>
     </row>
     <row r="509" ht="18" customHeight="1">

</xml_diff>